<commit_message>
Grouped inventory with committee and room-manager confirmation
Inventory now mirrors the school's "Data_Thietbi" list: equipment rows
with the same asset code, description and location are grouped and
their quantities summed. The inventory committee enters counted
quantity and condition, then "Xác nhận kiểm kê" upserts the group rows
(status, date, round). Room managers review and confirm or dispute the
result, which sets the confirmation status and date. Report shows
checked/confirmed rooms and missing/extra counts; the Excel template
for the inventory list follows the new columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JWuJVkZ8QmJV6ZRpzrxWrn
</commit_message>
<xml_diff>
--- a/templates/3_DieuChuyen.xlsx
+++ b/templates/3_DieuChuyen.xlsx
@@ -670,7 +670,11 @@
           <t>Số (Number)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Số lượng sổ sách = tổng thiết bị cùng Mã tài sản + Đặc điểm + Nơi sử dụng</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>